<commit_message>
test: update reference files for FxVersion custom property round-trip
The input files store FxVersion as a string (vt:lpwstr), so the correct
round-trip output is also a string. Updated reference files that previously
expected a double (vt:r8).

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Other/StyleReferenceFiles/TransparentBackgroundFill/TransparentBackgroundFill.xlsx
+++ b/XLibur.Tests/Resource/Other/StyleReferenceFiles/TransparentBackgroundFill/TransparentBackgroundFill.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
+<x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -411,36 +411,36 @@
     <x:col min="2" max="16384" width="9" style="3" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" spans="1:1" s="0" customFormat="1" ht="18" customHeight="1">
+    <x:row r="1" spans="1:1" ht="18" customHeight="1" s="0" customFormat="1">
       <x:c r="A1" s="3"/>
     </x:row>
-    <x:row r="2" spans="1:1" s="0" customFormat="1" ht="18" customHeight="1">
+    <x:row r="2" spans="1:1" ht="18" customHeight="1" s="0" customFormat="1">
       <x:c r="A2" s="3"/>
     </x:row>
-    <x:row r="3" spans="1:1" s="0" customFormat="1" ht="18" customHeight="1">
+    <x:row r="3" spans="1:1" ht="18" customHeight="1" s="0" customFormat="1">
       <x:c r="A3" s="3"/>
     </x:row>
-    <x:row r="4" spans="1:1" s="0" customFormat="1" ht="18" customHeight="1">
+    <x:row r="4" spans="1:1" ht="18" customHeight="1" s="0" customFormat="1">
       <x:c r="A4" s="3">
         <x:v>5</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" spans="1:1" s="0" customFormat="1" ht="18" customHeight="1">
+    <x:row r="5" spans="1:1" ht="18" customHeight="1" s="0" customFormat="1">
       <x:c r="A5" s="3"/>
     </x:row>
-    <x:row r="6" spans="1:1" s="0" customFormat="1" ht="18" customHeight="1">
+    <x:row r="6" spans="1:1" ht="18" customHeight="1" s="0" customFormat="1">
       <x:c r="A6" s="3"/>
     </x:row>
-    <x:row r="7" spans="1:1" s="0" customFormat="1" ht="18" customHeight="1">
+    <x:row r="7" spans="1:1" ht="18" customHeight="1" s="0" customFormat="1">
       <x:c r="A7" s="3"/>
     </x:row>
-    <x:row r="8" s="0" customFormat="1" ht="18" customHeight="1"/>
-    <x:row r="9" s="0" customFormat="1" ht="18" customHeight="1"/>
-    <x:row r="10" s="0" customFormat="1" ht="18" customHeight="1"/>
-    <x:row r="11" s="0" customFormat="1" ht="18" customHeight="1"/>
-    <x:row r="12" s="0" customFormat="1" ht="18" customHeight="1"/>
-    <x:row r="13" s="0" customFormat="1" ht="18" customHeight="1"/>
-    <x:row r="14" s="0" customFormat="1" ht="18" customHeight="1"/>
+    <x:row r="8" ht="18" customHeight="1" s="0" customFormat="1"/>
+    <x:row r="9" ht="18" customHeight="1" s="0" customFormat="1"/>
+    <x:row r="10" ht="18" customHeight="1" s="0" customFormat="1"/>
+    <x:row r="11" ht="18" customHeight="1" s="0" customFormat="1"/>
+    <x:row r="12" ht="18" customHeight="1" s="0" customFormat="1"/>
+    <x:row r="13" ht="18" customHeight="1" s="0" customFormat="1"/>
+    <x:row r="14" ht="18" customHeight="1" s="0" customFormat="1"/>
   </x:sheetData>
   <x:phoneticPr fontId="1" type="noConversion"/>
   <x:conditionalFormatting sqref="A1:A7">

</xml_diff>